<commit_message>
DD-korten: ett per köpt fastighet, effekten följer fyndet
DD-leken använder nu händelsekortens effektkoder (dolda brickor, underhållsvarning,
engångsbelopp, sällsynt direkt ±1 DN/energiklass) i stället för bara plus/minus.
Nya koder direkt_ek_plus/minus. Rättelse: breda FC-typer är inte yieldspåren.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_DD.xlsx
+++ b/kortdata/F_DD.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,6 +441,8 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,15 +463,25 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Synlig</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Värde</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Rubrik</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Beskrivning</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Antal exemplar</t>
         </is>
@@ -486,20 +498,26 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>direkt_dn_plus</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Ankarhyresgäst med långt avtal</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>En stabil hyresgäst har tio år kvar på kontraktet med full indexering.</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>En stabil hyresgäst har tio år kvar på kontraktet med full indexering. +1 DN direkt.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -514,20 +532,30 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>engangskassa_plus</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Outnyttjad byggrätt</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Detaljplanen medger fler kvadratmeter än vad som är byggt.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Detaljplanen medger fler kvadratmeter än vad som är byggt. Byggrätten säljs: +5 Mkr vid nästa marknad.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -542,20 +570,26 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Taket nylagt med garanti</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Yttertaket lades om för två år sedan med 25 års garanti.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -570,20 +604,26 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>Stambyte nyligen klart</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Stammar och våtrum renoverades i fjol. Underhållsbehovet är lågt de närmaste åren.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -598,20 +638,26 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Hyrorna ligger över snitt</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Indexklausulerna är strikta och hyrorna redan höjda till marknadsnivå.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -626,20 +672,26 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>Vakans redan uthyrd</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Lokalen som stod tom i prospektet har fått ny hyresgäst.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -654,20 +706,26 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>energi_plus</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>Miljöcertifiering på plats</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Fastigheten har giltig Miljöbyggnad Silver, vilket lockar fler hyresgäster.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -682,20 +740,26 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>Underhållsplanen har följts</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Säljaren har skött löpande underhåll noggrant. Inga eftersläpningar hittas.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -710,20 +774,26 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>energi_plus</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Solceller ger extra intäkt</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Taket har solceller som säljer överskottsel till nätet.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -738,20 +808,30 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>engangskassa_plus</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>Servitut gynnar fastigheten</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Grannfastigheten betalar för att nyttja garageinfarten.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="n">
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Grannfastigheten betalar för att nyttja garageinfarten. +2 Mkr vid nästa marknad.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -766,20 +846,26 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>Kö av intressenter till lediga lägenheter</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Bostadskön är lång och vakansgraden nästan obefintlig.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -794,20 +880,26 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Fasaden nyrenoverad</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Fönster och fasad byttes för tre år sedan. Inget akut underhåll krävs.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="H13" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -822,20 +914,26 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>Förråd och parkering efterfrågas</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Outhyrda extraytor har fler intressenter än platser.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="H14" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -850,20 +948,26 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>energi_plus</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>Bergvärme sänker driftkostnaden</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Fastigheten värms med bergvärme, vilket ger lägre energikostnad än väntat.</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="H15" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -878,20 +982,30 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>engangskassa_plus</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Fiberavtal ger löpande intäkt</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Ett nätbolag hyr in sig i teknikutrymmet och betalar årlig avgift.</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="n">
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Ett nätbolag hyr in sig i teknikutrymmet och betalar årlig avgift. +2 Mkr vid nästa marknad.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -906,20 +1020,30 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>dd_plus</t>
+          <t>engangskassa_plus</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>Byggrätt för vindsinredning</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Outnyttjad vind kan byggas om till fler lägenheter enligt gällande plan.</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="n">
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Outnyttjad vind kan byggas om till fler lägenheter enligt gällande plan. Byggrätten säljs: +3 Mkr vid nästa marknad.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -934,20 +1058,30 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Fuktskada i bjälklag</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Fukt har trängt in via en otät genomföring och skadat bärande konstruktion.</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="n">
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Fukt har trängt in via en otät genomföring och skadat bärande konstruktion. Underhållsvarning: 4 Mkr att röja.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -962,20 +1096,30 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>engangskassa_minus</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
           <t>Förorenad mark under garage</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Miljöprov visar olja och tungmetaller i marken.</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="n">
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Miljöprov visar olja och tungmetaller i marken. Sanering: −5 Mkr vid nästa marknad.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -990,20 +1134,30 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>engangskassa_minus</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
           <t>Asbest i ventilationskanaler</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Äldre ventilationskanaler innehåller asbest som måste saneras.</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="n">
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Äldre ventilationskanaler innehåller asbest som måste saneras. Sanering: −4 Mkr vid nästa marknad.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1018,20 +1172,26 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>energi_minus</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
           <t>Ventilationen underdimensionerad</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Anläggningen klarar inte dagens luftflödeskrav och måste byggas om.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1046,20 +1206,30 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
           <t>Taket eftersatt</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Yttertaket har nått slutet av sin livslängd och läcker vid kraftigt regn.</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="n">
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Yttertaket har nått slutet av sin livslängd och läcker vid kraftigt regn. Underhållsvarning: 3 Mkr att röja.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1074,20 +1244,30 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>engangskassa_minus</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
           <t>Radonhalt över gränsvärde</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Mätning visar förhöjd radonhalt. Radonsug krävs.</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="n">
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Mätning visar förhöjd radonhalt. Radonsug krävs. Radonsug: −2 Mkr vid nästa marknad.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1102,20 +1282,30 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
           <t>Hissen ej tillgänglighetsanpassad</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Hissen uppfyller inte dagens krav och behöver bytas ut.</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="n">
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Hissen uppfyller inte dagens krav och behöver bytas ut. Underhållsvarning: 3 Mkr att röja.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1130,20 +1320,30 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>engangskassa_minus</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
           <t>Brandskyddet brister i garage</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Sprinkler och brandlarm saknas på garageplanet.</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="n">
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Sprinkler och brandlarm saknas på garageplanet. −3 Mkr vid nästa marknad.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1158,20 +1358,30 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
           <t>Fasaden vittrar</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Tegelfogarna är nedslitna och behöver helfogas.</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="n">
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Tegelfogarna är nedslitna och behöver helfogas. Underhållsvarning: 3 Mkr att röja.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1186,20 +1396,26 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
           <t>Dolt servitut belastar fastigheten</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Grannen har rätt att nyttja infarten utan ersättning.</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="H27" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1214,20 +1430,26 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
           <t>Föråldrade hyresavtal</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Flera avtal saknar indexklausul och ligger under marknadshyra.</t>
         </is>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1242,20 +1464,26 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>direkt_dn_minus</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
           <t>Vakans dold i prospektet</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Säljaren har inte redovisat att en våning stått tom i ett halvår.</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="n">
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Säljaren har inte redovisat att en våning stått tom i ett halvår. −1 DN direkt.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1270,20 +1498,26 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
           <t>Indexklausul saknas i avtal</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Tre kommersiella hyresgäster har kontrakt utan uppräkning.</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="H30" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1298,20 +1532,30 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
           <t>Stammar i dåligt skick</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Rörstammarna är gamla och riskerar läckage inom kort.</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="n">
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Rörstammarna är gamla och riskerar läckage inom kort. Underhållsvarning: 4 Mkr att röja.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1326,20 +1570,26 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
           <t>Fuktskada i garage</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Dränering saknas och källarplanet står fuktigt vid regn.</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="H32" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1354,20 +1604,30 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>engangskassa_minus</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
           <t>Olovlig inredning upptäcks</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>En vind har inretts till bostad utan bygglov.</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="n">
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>En vind har inretts till bostad utan bygglov. Återställning: −2 Mkr vid nästa marknad.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1382,20 +1642,26 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
           <t>Tvist med hyresgäst pågår</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>En hyresgäst har stämt fastighetsägaren för uteblivet underhåll.</t>
         </is>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="H34" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1410,20 +1676,26 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>dd_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
+          <t>nej</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
           <t>Dåligt fungerande dränering</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>Marken runt grunden håller kvar vatten och riskerar fuktskador.</t>
         </is>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="H35" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1438,20 +1710,26 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>dd_ek</t>
+          <t>direkt_ek_minus</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
           <t>Energiklassen sämre än uppgiven</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Ny energideklaration visar lägre klass än vad säljaren angav.</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="n">
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Ny energideklaration visar lägre klass än vad säljaren angav. −1 energiklass direkt.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1466,20 +1744,26 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>dd_ek</t>
+          <t>direkt_ek_plus</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
           <t>Energiprestandan bättre än väntat</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Tilläggsisolering och nya fönster ger bättre energiklass än deklarerat.</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="n">
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Tilläggsisolering och nya fönster ger bättre energiklass än deklarerat. +1 energiklass direkt.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2106,7 +2390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2206,34 +2490,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rubrik</t>
+          <t>Synlig</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rubrik</t>
+          <t>Synlig</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nej</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Korttext</t>
+          <t>Mekanik — ändras bara genom design</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Beskrivning</t>
+          <t>Värde</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Beskrivning</t>
+          <t>Värde</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2243,27 +2527,71 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Korttext</t>
+          <t>Mekanik — ändras bara genom design</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Rubrik</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rubrik</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Korttext</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Beskrivning</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Beskrivning</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Korttext</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Antal exemplar</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Nej</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Per spel</t>
         </is>

</xml_diff>

<commit_message>
Inga kort ger kostnader eller pengar – bara påverkan på driftnettot
Regeländring (Niklas). I kortdata/ (källan):
- Händelsekort (13) och DD-kort (9) med engångsbelopp ger i stället en dold
  plus- eller minusbricka på fastigheten; texter med belopp omskrivna.
- Kvartalskorten 'varje ägare betalar X Mkr' (4) ger en dold minusbricka på
  varje fastighet av typen (ny effekt typbred_dolt_minus).
Trycktexterna (kortmallar) följer med, och underhållsvarningen säger att den
tas bort med kort. Balansen i BALANS.md; tryckfilerna behöver byggas om.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_DD.xlsx
+++ b/kortdata/F_DD.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -540,11 +540,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Outnyttjad byggrätt</t>
@@ -552,7 +548,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Detaljplanen medger fler kvadratmeter än vad som är byggt. Byggrätten säljs: +5 Mkr vid nästa marknad.</t>
+          <t>Detaljplanen medger fler kvadratmeter än vad som är byggt. Dold plusbricka på fastigheten.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -808,7 +804,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -816,11 +812,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Servitut gynnar fastigheten</t>
@@ -828,7 +820,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Grannfastigheten betalar för att nyttja garageinfarten. +2 Mkr vid nästa marknad.</t>
+          <t>Grannfastigheten betalar för att nyttja garageinfarten. Dold plusbricka på fastigheten.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -982,7 +974,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -990,11 +982,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Fiberavtal ger löpande intäkt</t>
@@ -1002,7 +990,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Ett nätbolag hyr in sig i teknikutrymmet och betalar årlig avgift. +2 Mkr vid nästa marknad.</t>
+          <t>Ett nätbolag hyr in sig i teknikutrymmet och betalar årlig avgift. Dold plusbricka på fastigheten.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1020,7 +1008,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_plus</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1028,11 +1016,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Byggrätt för vindsinredning</t>
@@ -1040,7 +1024,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Outnyttjad vind kan byggas om till fler lägenheter enligt gällande plan. Byggrätten säljs: +3 Mkr vid nästa marknad.</t>
+          <t>Outnyttjad vind kan byggas om till fler lägenheter enligt gällande plan. Dold plusbricka på fastigheten.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1096,7 +1080,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1104,11 +1088,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+      <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Förorenad mark under garage</t>
@@ -1116,7 +1096,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Miljöprov visar olja och tungmetaller i marken. Sanering: −5 Mkr vid nästa marknad.</t>
+          <t>Miljöprov visar olja och tungmetaller i marken. Dold minusbricka på fastigheten.</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1134,7 +1114,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1142,11 +1122,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+      <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Asbest i ventilationskanaler</t>
@@ -1154,7 +1130,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Äldre ventilationskanaler innehåller asbest som måste saneras. Sanering: −4 Mkr vid nästa marknad.</t>
+          <t>Äldre ventilationskanaler innehåller asbest som måste saneras. Dold minusbricka på fastigheten.</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
@@ -1244,7 +1220,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1252,11 +1228,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Radonhalt över gränsvärde</t>
@@ -1264,7 +1236,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Mätning visar förhöjd radonhalt. Radonsug krävs. Radonsug: −2 Mkr vid nästa marknad.</t>
+          <t>Mätning visar förhöjd radonhalt. Radonsug krävs. Dold minusbricka på fastigheten.</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
@@ -1320,7 +1292,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1328,11 +1300,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Brandskyddet brister i garage</t>
@@ -1340,7 +1308,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Sprinkler och brandlarm saknas på garageplanet. −3 Mkr vid nästa marknad.</t>
+          <t>Sprinkler och brandlarm saknas på garageplanet. Dold minusbricka på fastigheten.</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
@@ -1604,7 +1572,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_minus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1612,11 +1580,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Olovlig inredning upptäcks</t>
@@ -1624,7 +1588,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>En vind har inretts till bostad utan bygglov. Återställning: −2 Mkr vid nästa marknad.</t>
+          <t>En vind har inretts till bostad utan bygglov. Dold minusbricka på fastigheten.</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">

</xml_diff>

<commit_message>
Korttexter inför omtrycket: DD utan röjningskostnad, FC Skölden och Bostadsveteranen
- F_DD: fem underhållsvarningar sa 'X Mkr att röja' → 'Underhållsvarning – tas bort med kort'.
- F_FC: Sköldens juniortext kortad (krockade med foten); Bostadsveteranens seniortext säger
  vad som gäller två gånger per kvartal.
- kort.css: typetiketten håller ihop när den bryts (Skölden: lokal, kontor, förskola).
Tryckfilerna (tryck/ut, ej i git) byggda om: 8 lekar, 734 sidor, 0 krockar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_DD.xlsx
+++ b/kortdata/F_DD.xlsx
@@ -1062,7 +1062,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Fukt har trängt in via en otät genomföring och skadat bärande konstruktion. Underhållsvarning: 4 Mkr att röja.</t>
+          <t>Fukt har trängt in via en otät genomföring och skadat bärande konstruktion. Underhållsvarning – tas bort med kort.</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Yttertaket har nått slutet av sin livslängd och läcker vid kraftigt regn. Underhållsvarning: 3 Mkr att röja.</t>
+          <t>Yttertaket har nått slutet av sin livslängd och läcker vid kraftigt regn. Underhållsvarning – tas bort med kort.</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Hissen uppfyller inte dagens krav och behöver bytas ut. Underhållsvarning: 3 Mkr att röja.</t>
+          <t>Hissen uppfyller inte dagens krav och behöver bytas ut. Underhållsvarning – tas bort med kort.</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Tegelfogarna är nedslitna och behöver helfogas. Underhållsvarning: 3 Mkr att röja.</t>
+          <t>Tegelfogarna är nedslitna och behöver helfogas. Underhållsvarning – tas bort med kort.</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Rörstammarna är gamla och riskerar läckage inom kort. Underhållsvarning: 4 Mkr att röja.</t>
+          <t>Rörstammarna är gamla och riskerar läckage inom kort. Underhållsvarning – tas bort med kort.</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">

</xml_diff>